<commit_message>
Exp3: GRPO_LA0 finished (10 iters) + results/docs update
GRPO_LA0 ran to completion (model states 0-10, re-scored on full battery).
Key finding: GRPO peaks at iter 8 (Q1Q2 4.08) then REGRESSES (iter9 3.81,
iter10 3.75) while PTO climbs stably to 4.26 — so the prior "near-tie at
iter 8" flips to PTO ahead at the matched 10-iter endpoint (paired PTO-GRPO
+0.51, dz +0.73, Holm p<0.001). Mechanism (confirmed in iter-10 convs on the
same resistant persona): GRPO collapses into pure sycophancy (0.13 q/turn,
3.61 praise-words/turn) and never delivers advice; PTO drifts toward
affirmation too but converges to concrete steps (0.50 q/turn, 1.02 praise).

- Regenerated eval/headline/stats figures + tables for the finished GRPO arm.
- Updated root + Exp3 CLAUDE.md (status, "Eval results so far", drift bullet).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Exp3_PTO_GRPO/eda/results/tables/eval/eval.xlsx
+++ b/Exp3_PTO_GRPO/eda/results/tables/eval/eval.xlsx
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,6 +994,70 @@
       </c>
       <c r="J10" t="n">
         <v>0.231</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>6.438</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3.958</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.083</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.583</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.188</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4.292</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.158</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4.115</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.021</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.979</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.375</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.435</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>